<commit_message>
Update web and add complete mobile app with FAST brand styling and features
</commit_message>
<xml_diff>
--- a/frontend/public/sample_candidate_emails.xlsx
+++ b/frontend/public/sample_candidate_emails.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Candidate_Emails" sheetId="1" r:id="rId1"/>
+    <sheet name="Candidates" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,119 +397,347 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A21"/>
-  <cols>
-    <col min="1" max="1" width="35.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D24"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Email</v>
       </c>
+      <c r="B1" t="str">
+        <v>Candidate Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>City</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Has Resume in Portal</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>rahul.sharma@fastcareers.in</v>
       </c>
+      <c r="B2" t="str">
+        <v>Rahul Sharma</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Mumbai</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>priya.patel@fastcareers.in</v>
       </c>
+      <c r="B3" t="str">
+        <v>Priya Patel</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Ahmedabad</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>amit.verma@fastcareers.in</v>
       </c>
+      <c r="B4" t="str">
+        <v>Amit Verma</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Delhi</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>neha.singh@fastcareers.in</v>
       </c>
+      <c r="B5" t="str">
+        <v>Neha Singh</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Bengaluru</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
         <v>vikram.malhotra@fastcareers.in</v>
       </c>
+      <c r="B6" t="str">
+        <v>Vikram Malhotra</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>ananya.gupta@fastcareers.in</v>
       </c>
+      <c r="B7" t="str">
+        <v>Ananya Gupta</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>rohan.mehta@fastcareers.in</v>
       </c>
+      <c r="B8" t="str">
+        <v>Rohan Mehta</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Hyderabad</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
         <v>sneha.reddy@fastcareers.in</v>
       </c>
+      <c r="B9" t="str">
+        <v>Sneha Reddy</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Chennai</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
         <v>aditya.joshi@fastcareers.in</v>
       </c>
+      <c r="B10" t="str">
+        <v>Aditya Joshi</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Jaipur</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
         <v>pooja.nair@fastcareers.in</v>
       </c>
+      <c r="B11" t="str">
+        <v>Pooja Nair</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Kochi</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
         <v>kunal.kapoor@fastcareers.in</v>
       </c>
+      <c r="B12" t="str">
+        <v>Kunal Kapoor</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Gurugram</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
         <v>divya.saxena@fastcareers.in</v>
       </c>
+      <c r="B13" t="str">
+        <v>Divya Saxena</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Noida</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Yes</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>suresh.iyer@fastcareers.in</v>
+        <v>manish.agarwal@fastcareers.in</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Manish Agarwal</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Indore</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Yes</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>meera.kulkarni@fastcareers.in</v>
+        <v>ritu.jain@fastcareers.in</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Ritu Jain</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Chandigarh</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Yes</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>deepak.agarwal@fastcareers.in</v>
+        <v>saurabh.mishra@fastcareers.in</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Saurabh Mishra</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Lucknow</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Yes</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ritu.chawla@fastcareers.in</v>
+        <v>tanvi.kulkarni@fastcareers.in</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Tanvi Kulkarni</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Mumbai</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Yes</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>gaurav.bhatia@fastcareers.in</v>
+        <v>deepesh.bansal@fastcareers.in</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Deepesh Bansal</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Surat</v>
+      </c>
+      <c r="D18" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>tanvi.deshmukh@fastcareers.in</v>
+        <v>kavita.choudhary@fastcareers.in</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Kavita Choudhary</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Bhopal</v>
+      </c>
+      <c r="D19" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>nitin.singhania@fastcareers.in</v>
+        <v>harshit.goyal@fastcareers.in</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Harshit Goyal</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Ludhiana</v>
+      </c>
+      <c r="D20" t="str">
+        <v>No</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>shreya.banerjee@fastcareers.in</v>
+        <v>meenakshi.sundaram@fastcareers.in</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Meenakshi Sundaram</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Coimbatore</v>
+      </c>
+      <c r="D21" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>unknown.candidate1@external.com</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Unknown Candidate 1</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Mumbai</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Not in DB</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>notfound.tester@gmail.com</v>
+      </c>
+      <c r="B23" t="str">
+        <v>NotFound Tester</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Delhi</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Not in DB</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>RAHUL.SHARMA@FASTCAREERS.IN</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Rahul Sharma (Uppercase Duplicate)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Mumbai</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Duplicate</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>